<commit_message>
Update NY gaming data - Fri Sep  4 15:40:49 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_analysis.xlsx
+++ b/ny_gaming_analysis.xlsx
@@ -499,10 +499,10 @@
         <v>149527600</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>5527466</v>
       </c>
       <c r="G2" t="n">
-        <v>146777768</v>
+        <v>146777769</v>
       </c>
       <c r="H2" t="n">
         <v>52848942</v>
@@ -511,10 +511,10 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>8585058</v>
       </c>
       <c r="K2" t="n">
-        <v>406173189</v>
+        <v>420285714</v>
       </c>
     </row>
     <row r="3">
@@ -9069,16 +9069,16 @@
         <v>2727869</v>
       </c>
       <c r="D2" t="n">
-        <v>2177229.24</v>
+        <v>2177229</v>
       </c>
       <c r="E2" t="n">
         <v>12079306</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>360457</v>
       </c>
       <c r="G2" t="n">
-        <v>15874316.7285</v>
+        <v>15874317</v>
       </c>
       <c r="H2" t="n">
         <v>5061346</v>
@@ -9087,10 +9087,10 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>755239</v>
       </c>
       <c r="K2" t="n">
-        <v>38184968.9685</v>
+        <v>39300665</v>
       </c>
     </row>
     <row r="3">
@@ -17645,22 +17645,26 @@
         <v>0.09356311131492324</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.08508656539005444</v>
+        <v>0.08508655601080521</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.08078311963811363</v>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" s="2" t="n">
+        <v>0.06521197959426617</v>
+      </c>
       <c r="G2" s="2" t="n">
-        <v>0.1081520515320821</v>
+        <v>0.1081520526449751</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0.09577005344780601</v>
       </c>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" s="2" t="n">
+        <v>0.08797133344934886</v>
+      </c>
       <c r="K2" s="2" t="n">
-        <v>0.09401154483512696</v>
+        <v>0.09350940013154956</v>
       </c>
     </row>
     <row r="3">
@@ -25957,20 +25961,20 @@
         <v>-0.1010761282789343</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.437537135242751</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-0.03760194506240455</v>
+        <v>-0.03760193850556648</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>-0.6376083250515292</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.1799154091086376</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>-0.2722330102215654</v>
+        <v>-0.2469466788841642</v>
       </c>
     </row>
     <row r="3">
@@ -33335,26 +33339,26 @@
         <v>-0.3728721055151972</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>-0.3828953192280571</v>
+        <v>-0.3828953872526456</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>-0.3949443291756074</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.590415837173998</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-0.2668612214317583</v>
+        <v>-0.2668612088928135</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>-0.6580329896893286</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.3767138041024837</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>-0.4269964961373741</v>
+        <v>-0.4102543655932193</v>
       </c>
     </row>
     <row r="3">

</xml_diff>